<commit_message>
Regenerate stale security readiness reports
Co-authored-by: WGLewis0721 <22523406+WGLewis0721@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/implementation/security-readiness/apps/studigo/generated/security-readiness.xlsx
+++ b/implementation/security-readiness/apps/studigo/generated/security-readiness.xlsx
@@ -2235,7 +2235,7 @@
 **How to verify:**
 1. Sample production logs and telemetry for content and credentials.
 **Suggested fix:** Audit logs/telemetry payloads and enforce redaction/minimization.
-**Evidence so far:** implementation/AI_ENGINEERING_HARDENING_PLAN.md
+**Evidence so far:** implementation/ENGINEERING_PLAN.md
 **Evidence required to close:** Logging policy and sampled traces.
 **Standards:** OWASP Logging Cheat Sheet, OWASP LLM02:2025</t>
         </is>
@@ -3035,7 +3035,7 @@
 **How to verify:**
 1. Find yesterday's cost by operation and the top-spending user.
 **Suggested fix:** Add privacy-conscious AI tracing and operation/user/global budgets.
-**Evidence so far:** evals/rag/README.md, implementation/AI_ENGINEERING_HARDENING_PLAN.md
+**Evidence so far:** evals/rag/README.md, implementation/ENGINEERING_PLAN.md
 **Evidence required to close:** Telemetry schema/dashboard/query evidence.
 **Standards:** OWASP LLM10:2025, NIST AI RMF MANAGE 4</t>
         </is>
@@ -3564,7 +3564,7 @@
 **How to verify:**
 1. Pick a stored answer and identify the exact model and prompt that produced it.
 **Suggested fix:** Adopt one AI trace/version envelope across all provider calls.
-**Evidence so far:** packages/ai/src/coach.ts, implementation/AI_ENGINEERING_HARDENING_PLAN.md
+**Evidence so far:** packages/ai/src/coach.ts, implementation/ENGINEERING_PLAN.md
 **Evidence required to close:** Versioned configs/traces and reproducibility test.
 **Standards:** NIST AI RMF MEASURE 2, NIST AI 600-1: Information Integrity</t>
         </is>
@@ -3653,7 +3653,7 @@
 1. Compare the inventory with deployed services, environment variables and provider dashboards.
 2. Trace one sensitive record from intake to deletion and confirm every hop is documented.
 **Suggested fix:** Create security threat model/data-flow map and keep it synchronized with production components.
-**Evidence so far:** docs/ARCHITECTURE.md, implementation/AI_SOFTWARE_ENGINEERING_WALKTHROUGH.md
+**Evidence so far:** docs/ARCHITECTURE.md, ENGINEERING.md
 **Evidence required to close:** Current data-flow/trust-boundary diagram and component inventory.
 **Standards:** NIST SSDF PO.1, NIST AI RMF MAP 1, OWASP Top 10:2021 A04</t>
         </is>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t xml:space="preserve">docs/ARCHITECTURE.md|implementation/AI_SOFTWARE_ENGINEERING_WALKTHROUGH.md</t>
+          <t xml:space="preserve">docs/ARCHITECTURE.md|ENGINEERING.md</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -8721,7 +8721,7 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t xml:space="preserve">packages/ai/src/coach.ts|implementation/AI_ENGINEERING_HARDENING_PLAN.md</t>
+          <t xml:space="preserve">packages/ai/src/coach.ts|implementation/ENGINEERING_PLAN.md</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
@@ -8860,7 +8860,7 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t xml:space="preserve">evals/rag/README.md|implementation/AI_ENGINEERING_HARDENING_PLAN.md</t>
+          <t xml:space="preserve">evals/rag/README.md|implementation/ENGINEERING_PLAN.md</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
@@ -10293,7 +10293,7 @@
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t xml:space="preserve">implementation/AI_ENGINEERING_HARDENING_PLAN.md</t>
+          <t xml:space="preserve">implementation/ENGINEERING_PLAN.md</t>
         </is>
       </c>
       <c r="W43" t="inlineStr">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">implementation/AI_SOFTWARE_ENGINEERING_WALKTHROUGH.md</t>
+          <t xml:space="preserve">ENGINEERING.md</t>
         </is>
       </c>
     </row>
@@ -14949,7 +14949,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">implementation/AI_ENGINEERING_HARDENING_PLAN.md</t>
+          <t xml:space="preserve">implementation/ENGINEERING_PLAN.md</t>
         </is>
       </c>
     </row>
@@ -15003,7 +15003,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t xml:space="preserve">implementation/AI_ENGINEERING_HARDENING_PLAN.md</t>
+          <t xml:space="preserve">implementation/ENGINEERING_PLAN.md</t>
         </is>
       </c>
     </row>
@@ -15570,7 +15570,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t xml:space="preserve">implementation/AI_ENGINEERING_HARDENING_PLAN.md</t>
+          <t xml:space="preserve">implementation/ENGINEERING_PLAN.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: refresh security reports after the plan rename
The generated evidence still cited the removed hardening plan and walkthrough. Status is unchanged: not ready, 29 blockers.
</commit_message>
<xml_diff>
--- a/implementation/security-readiness/apps/studigo/generated/security-readiness.xlsx
+++ b/implementation/security-readiness/apps/studigo/generated/security-readiness.xlsx
@@ -2235,7 +2235,7 @@
 **How to verify:**
 1. Sample production logs and telemetry for content and credentials.
 **Suggested fix:** Audit logs/telemetry payloads and enforce redaction/minimization.
-**Evidence so far:** implementation/AI_ENGINEERING_HARDENING_PLAN.md
+**Evidence so far:** implementation/ENGINEERING_PLAN.md
 **Evidence required to close:** Logging policy and sampled traces.
 **Standards:** OWASP Logging Cheat Sheet, OWASP LLM02:2025</t>
         </is>
@@ -3035,7 +3035,7 @@
 **How to verify:**
 1. Find yesterday's cost by operation and the top-spending user.
 **Suggested fix:** Add privacy-conscious AI tracing and operation/user/global budgets.
-**Evidence so far:** evals/rag/README.md, implementation/AI_ENGINEERING_HARDENING_PLAN.md
+**Evidence so far:** evals/rag/README.md, implementation/ENGINEERING_PLAN.md
 **Evidence required to close:** Telemetry schema/dashboard/query evidence.
 **Standards:** OWASP LLM10:2025, NIST AI RMF MANAGE 4</t>
         </is>
@@ -3564,7 +3564,7 @@
 **How to verify:**
 1. Pick a stored answer and identify the exact model and prompt that produced it.
 **Suggested fix:** Adopt one AI trace/version envelope across all provider calls.
-**Evidence so far:** packages/ai/src/coach.ts, implementation/AI_ENGINEERING_HARDENING_PLAN.md
+**Evidence so far:** packages/ai/src/coach.ts, implementation/ENGINEERING_PLAN.md
 **Evidence required to close:** Versioned configs/traces and reproducibility test.
 **Standards:** NIST AI RMF MEASURE 2, NIST AI 600-1: Information Integrity</t>
         </is>
@@ -3653,7 +3653,7 @@
 1. Compare the inventory with deployed services, environment variables and provider dashboards.
 2. Trace one sensitive record from intake to deletion and confirm every hop is documented.
 **Suggested fix:** Create security threat model/data-flow map and keep it synchronized with production components.
-**Evidence so far:** docs/ARCHITECTURE.md, implementation/AI_SOFTWARE_ENGINEERING_WALKTHROUGH.md
+**Evidence so far:** docs/ARCHITECTURE.md, ENGINEERING.md
 **Evidence required to close:** Current data-flow/trust-boundary diagram and component inventory.
 **Standards:** NIST SSDF PO.1, NIST AI RMF MAP 1, OWASP Top 10:2021 A04</t>
         </is>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t xml:space="preserve">docs/ARCHITECTURE.md|implementation/AI_SOFTWARE_ENGINEERING_WALKTHROUGH.md</t>
+          <t xml:space="preserve">docs/ARCHITECTURE.md|ENGINEERING.md</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -8721,7 +8721,7 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t xml:space="preserve">packages/ai/src/coach.ts|implementation/AI_ENGINEERING_HARDENING_PLAN.md</t>
+          <t xml:space="preserve">packages/ai/src/coach.ts|implementation/ENGINEERING_PLAN.md</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
@@ -8860,7 +8860,7 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t xml:space="preserve">evals/rag/README.md|implementation/AI_ENGINEERING_HARDENING_PLAN.md</t>
+          <t xml:space="preserve">evals/rag/README.md|implementation/ENGINEERING_PLAN.md</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
@@ -10293,7 +10293,7 @@
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t xml:space="preserve">implementation/AI_ENGINEERING_HARDENING_PLAN.md</t>
+          <t xml:space="preserve">implementation/ENGINEERING_PLAN.md</t>
         </is>
       </c>
       <c r="W43" t="inlineStr">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">implementation/AI_SOFTWARE_ENGINEERING_WALKTHROUGH.md</t>
+          <t xml:space="preserve">ENGINEERING.md</t>
         </is>
       </c>
     </row>
@@ -14949,7 +14949,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">implementation/AI_ENGINEERING_HARDENING_PLAN.md</t>
+          <t xml:space="preserve">implementation/ENGINEERING_PLAN.md</t>
         </is>
       </c>
     </row>
@@ -15003,7 +15003,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t xml:space="preserve">implementation/AI_ENGINEERING_HARDENING_PLAN.md</t>
+          <t xml:space="preserve">implementation/ENGINEERING_PLAN.md</t>
         </is>
       </c>
     </row>
@@ -15570,7 +15570,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t xml:space="preserve">implementation/AI_ENGINEERING_HARDENING_PLAN.md</t>
+          <t xml:space="preserve">implementation/ENGINEERING_PLAN.md</t>
         </is>
       </c>
     </row>

</xml_diff>